<commit_message>
updated xlsx file handling for multi-sheet across multiple files
</commit_message>
<xml_diff>
--- a/datasets/excel tests/2 multi-single menu_items.xlsx
+++ b/datasets/excel tests/2 multi-single menu_items.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pmclu\Documents\2026 Summer\capstone\ai-dashboards\datasets\excel tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AAEFAA3D-FEBC-4BE3-A710-0BBAC14A0E71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{245D2785-5430-43F1-9BEC-6684FFDF0697}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" xr2:uid="{86CB8E09-F6C5-435B-B1E2-ECE3B98D75F7}"/>
+    <workbookView xWindow="6144" yWindow="7092" windowWidth="23040" windowHeight="13560" xr2:uid="{86CB8E09-F6C5-435B-B1E2-ECE3B98D75F7}"/>
   </bookViews>
   <sheets>
     <sheet name="2 multi-single menu_items" sheetId="1" r:id="rId1"/>
@@ -22,9 +22,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="40">
   <si>
-    <t>menu_item_id</t>
-  </si>
-  <si>
     <t>item_name</t>
   </si>
   <si>
@@ -140,6 +137,9 @@
   </si>
   <si>
     <t>Eggplant Parmesan</t>
+  </si>
+  <si>
+    <t>item_id</t>
   </si>
 </sst>
 </file>
@@ -1005,16 +1005,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -1022,10 +1022,10 @@
         <v>101</v>
       </c>
       <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
         <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
       </c>
       <c r="D2">
         <v>12.95</v>
@@ -1036,10 +1036,10 @@
         <v>102</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D3">
         <v>13.95</v>
@@ -1050,10 +1050,10 @@
         <v>103</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D4">
         <v>9</v>
@@ -1064,10 +1064,10 @@
         <v>104</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D5">
         <v>10.5</v>
@@ -1078,10 +1078,10 @@
         <v>105</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D6">
         <v>7</v>
@@ -1092,10 +1092,10 @@
         <v>106</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D7">
         <v>7</v>
@@ -1106,10 +1106,10 @@
         <v>107</v>
       </c>
       <c r="B8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" t="s">
         <v>11</v>
-      </c>
-      <c r="C8" t="s">
-        <v>12</v>
       </c>
       <c r="D8">
         <v>16.5</v>
@@ -1120,10 +1120,10 @@
         <v>108</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D9">
         <v>14.5</v>
@@ -1134,10 +1134,10 @@
         <v>109</v>
       </c>
       <c r="B10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D10">
         <v>17.95</v>
@@ -1148,10 +1148,10 @@
         <v>110</v>
       </c>
       <c r="B11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D11">
         <v>17.95</v>
@@ -1162,10 +1162,10 @@
         <v>111</v>
       </c>
       <c r="B12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D12">
         <v>11.95</v>
@@ -1176,10 +1176,10 @@
         <v>112</v>
       </c>
       <c r="B13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D13">
         <v>14.95</v>
@@ -1190,10 +1190,10 @@
         <v>113</v>
       </c>
       <c r="B14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C14" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D14">
         <v>5</v>
@@ -1204,10 +1204,10 @@
         <v>114</v>
       </c>
       <c r="B15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C15" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D15">
         <v>9</v>
@@ -1218,10 +1218,10 @@
         <v>115</v>
       </c>
       <c r="B16" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" t="s">
         <v>20</v>
-      </c>
-      <c r="C16" t="s">
-        <v>21</v>
       </c>
       <c r="D16">
         <v>11.95</v>
@@ -1232,10 +1232,10 @@
         <v>116</v>
       </c>
       <c r="B17" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D17">
         <v>13.95</v>
@@ -1246,10 +1246,10 @@
         <v>117</v>
       </c>
       <c r="B18" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D18">
         <v>12.95</v>
@@ -1260,10 +1260,10 @@
         <v>118</v>
       </c>
       <c r="B19" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C19" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D19">
         <v>14.95</v>
@@ -1274,10 +1274,10 @@
         <v>119</v>
       </c>
       <c r="B20" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C20" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D20">
         <v>11.95</v>
@@ -1288,10 +1288,10 @@
         <v>120</v>
       </c>
       <c r="B21" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C21" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D21">
         <v>13.95</v>
@@ -1302,10 +1302,10 @@
         <v>121</v>
       </c>
       <c r="B22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D22">
         <v>10.5</v>
@@ -1316,10 +1316,10 @@
         <v>122</v>
       </c>
       <c r="B23" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C23" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D23">
         <v>7</v>
@@ -1330,10 +1330,10 @@
         <v>123</v>
       </c>
       <c r="B24" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C24" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D24">
         <v>9</v>
@@ -1344,10 +1344,10 @@
         <v>124</v>
       </c>
       <c r="B25" t="s">
+        <v>29</v>
+      </c>
+      <c r="C25" t="s">
         <v>30</v>
-      </c>
-      <c r="C25" t="s">
-        <v>31</v>
       </c>
       <c r="D25">
         <v>14.5</v>
@@ -1358,10 +1358,10 @@
         <v>125</v>
       </c>
       <c r="B26" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C26" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D26">
         <v>17.95</v>
@@ -1372,10 +1372,10 @@
         <v>126</v>
       </c>
       <c r="B27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D27">
         <v>14.5</v>
@@ -1386,10 +1386,10 @@
         <v>127</v>
       </c>
       <c r="B28" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C28" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D28">
         <v>17.95</v>
@@ -1400,10 +1400,10 @@
         <v>128</v>
       </c>
       <c r="B29" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C29" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D29">
         <v>15.5</v>
@@ -1414,10 +1414,10 @@
         <v>129</v>
       </c>
       <c r="B30" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D30">
         <v>15.5</v>
@@ -1428,10 +1428,10 @@
         <v>130</v>
       </c>
       <c r="B31" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C31" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D31">
         <v>19.95</v>
@@ -1442,10 +1442,10 @@
         <v>131</v>
       </c>
       <c r="B32" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C32" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D32">
         <v>17.95</v>
@@ -1456,10 +1456,10 @@
         <v>132</v>
       </c>
       <c r="B33" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C33" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D33">
         <v>16.95</v>

</xml_diff>